<commit_message>
updated g sheets to copy 2025 to 2026. updated rating file for ref
</commit_message>
<xml_diff>
--- a/archive/LS_rating_apr.xlsx
+++ b/archive/LS_rating_apr.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaimin Khaw\Desktop\credit-rating-deploy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kaimin Khaw\Desktop\credit-rating-deploy\archive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD9E02B1-D2F3-441E-90A4-112B86A4FC96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBCDC6E-8E20-4A33-9061-82F1ABD84EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5484,7 +5484,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26FFD78D-BBF8-44CD-974B-54BFCD0DE856}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:I139"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5524,7 +5523,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -5554,7 +5553,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -5584,7 +5583,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -5614,7 +5613,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -5644,7 +5643,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -5674,7 +5673,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -5704,7 +5703,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -5734,7 +5733,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -5764,7 +5763,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -5794,7 +5793,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>35</v>
       </c>
@@ -5824,7 +5823,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>37</v>
       </c>
@@ -5854,7 +5853,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -5884,7 +5883,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>41</v>
       </c>
@@ -5914,7 +5913,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -5944,7 +5943,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>44</v>
       </c>
@@ -5974,7 +5973,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>48</v>
       </c>
@@ -6004,7 +6003,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>50</v>
       </c>
@@ -6034,7 +6033,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>52</v>
       </c>
@@ -6064,7 +6063,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -6094,7 +6093,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>55</v>
       </c>
@@ -6124,7 +6123,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>57</v>
       </c>
@@ -6154,7 +6153,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>58</v>
       </c>
@@ -6184,7 +6183,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>59</v>
       </c>
@@ -6214,7 +6213,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -6244,7 +6243,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -6274,7 +6273,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>68</v>
       </c>
@@ -6304,7 +6303,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>71</v>
       </c>
@@ -6364,7 +6363,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>77</v>
       </c>
@@ -6394,7 +6393,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>78</v>
       </c>
@@ -6424,7 +6423,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>80</v>
       </c>
@@ -6454,7 +6453,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>81</v>
       </c>
@@ -6484,7 +6483,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>82</v>
       </c>
@@ -6514,7 +6513,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>83</v>
       </c>
@@ -6544,7 +6543,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>84</v>
       </c>
@@ -6574,7 +6573,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>87</v>
       </c>
@@ -6604,7 +6603,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>88</v>
       </c>
@@ -6634,7 +6633,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>91</v>
       </c>
@@ -6664,7 +6663,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>92</v>
       </c>
@@ -6694,7 +6693,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>93</v>
       </c>
@@ -6724,7 +6723,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>94</v>
       </c>
@@ -6754,7 +6753,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>95</v>
       </c>
@@ -6784,7 +6783,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>96</v>
       </c>
@@ -6814,7 +6813,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>98</v>
       </c>
@@ -6844,7 +6843,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>100</v>
       </c>
@@ -6874,7 +6873,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>101</v>
       </c>
@@ -6904,7 +6903,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>102</v>
       </c>
@@ -6934,7 +6933,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>104</v>
       </c>
@@ -6964,7 +6963,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>105</v>
       </c>
@@ -6994,7 +6993,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>106</v>
       </c>
@@ -7024,7 +7023,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>109</v>
       </c>
@@ -7054,7 +7053,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>110</v>
       </c>
@@ -7084,7 +7083,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>111</v>
       </c>
@@ -7114,7 +7113,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>112</v>
       </c>
@@ -7174,7 +7173,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>114</v>
       </c>
@@ -7204,7 +7203,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>115</v>
       </c>
@@ -7234,7 +7233,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>116</v>
       </c>
@@ -7294,7 +7293,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>118</v>
       </c>
@@ -7324,7 +7323,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>119</v>
       </c>
@@ -7354,7 +7353,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>120</v>
       </c>
@@ -7384,7 +7383,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>121</v>
       </c>
@@ -7414,7 +7413,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>122</v>
       </c>
@@ -7444,7 +7443,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>123</v>
       </c>
@@ -7474,7 +7473,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>124</v>
       </c>
@@ -7504,7 +7503,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>125</v>
       </c>
@@ -7534,7 +7533,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>126</v>
       </c>
@@ -7564,7 +7563,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>127</v>
       </c>
@@ -7624,7 +7623,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>131</v>
       </c>
@@ -7654,7 +7653,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>132</v>
       </c>
@@ -7684,7 +7683,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>133</v>
       </c>
@@ -7714,7 +7713,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>134</v>
       </c>
@@ -7744,7 +7743,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>135</v>
       </c>
@@ -7774,7 +7773,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>136</v>
       </c>
@@ -7804,7 +7803,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>137</v>
       </c>
@@ -7834,7 +7833,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>138</v>
       </c>
@@ -7864,7 +7863,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>204</v>
       </c>
@@ -7885,7 +7884,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>139</v>
       </c>
@@ -7915,7 +7914,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>141</v>
       </c>
@@ -7945,7 +7944,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="83" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>142</v>
       </c>
@@ -7975,7 +7974,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>143</v>
       </c>
@@ -8005,7 +8004,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>144</v>
       </c>
@@ -8035,7 +8034,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="86" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>145</v>
       </c>
@@ -8065,7 +8064,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>146</v>
       </c>
@@ -8095,7 +8094,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>147</v>
       </c>
@@ -8125,7 +8124,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>148</v>
       </c>
@@ -8215,7 +8214,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>152</v>
       </c>
@@ -8245,7 +8244,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>153</v>
       </c>
@@ -8275,7 +8274,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>154</v>
       </c>
@@ -8305,7 +8304,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>155</v>
       </c>
@@ -8335,7 +8334,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>156</v>
       </c>
@@ -8365,7 +8364,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>157</v>
       </c>
@@ -8395,7 +8394,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>159</v>
       </c>
@@ -8455,7 +8454,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>162</v>
       </c>
@@ -8485,7 +8484,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>163</v>
       </c>
@@ -8545,7 +8544,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>165</v>
       </c>
@@ -8575,7 +8574,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>166</v>
       </c>
@@ -8605,7 +8604,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>167</v>
       </c>
@@ -8635,7 +8634,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>168</v>
       </c>
@@ -8665,7 +8664,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>169</v>
       </c>
@@ -8695,7 +8694,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>170</v>
       </c>
@@ -8725,7 +8724,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>171</v>
       </c>
@@ -8755,7 +8754,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>172</v>
       </c>
@@ -8785,7 +8784,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>173</v>
       </c>
@@ -8815,7 +8814,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>174</v>
       </c>
@@ -8845,7 +8844,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>175</v>
       </c>
@@ -8875,7 +8874,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>176</v>
       </c>
@@ -8905,7 +8904,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>177</v>
       </c>
@@ -8935,7 +8934,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>178</v>
       </c>
@@ -8965,7 +8964,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>179</v>
       </c>
@@ -8995,7 +8994,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>180</v>
       </c>
@@ -9025,7 +9024,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>181</v>
       </c>
@@ -9055,7 +9054,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>182</v>
       </c>
@@ -9085,7 +9084,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>183</v>
       </c>
@@ -9115,7 +9114,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>184</v>
       </c>
@@ -9145,7 +9144,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>185</v>
       </c>
@@ -9175,7 +9174,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>186</v>
       </c>
@@ -9205,7 +9204,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>187</v>
       </c>
@@ -9235,7 +9234,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>188</v>
       </c>
@@ -9265,7 +9264,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>189</v>
       </c>
@@ -9295,7 +9294,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>190</v>
       </c>
@@ -9325,7 +9324,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>191</v>
       </c>
@@ -9355,7 +9354,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>192</v>
       </c>
@@ -9385,7 +9384,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>193</v>
       </c>
@@ -9415,7 +9414,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="132" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>194</v>
       </c>
@@ -9475,7 +9474,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>196</v>
       </c>
@@ -9505,7 +9504,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>197</v>
       </c>
@@ -9535,7 +9534,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="136" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>198</v>
       </c>
@@ -9565,7 +9564,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>199</v>
       </c>
@@ -9595,7 +9594,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>200</v>
       </c>
@@ -9625,7 +9624,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>201</v>
       </c>
@@ -9656,21 +9655,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I139" xr:uid="{26FFD78D-BBF8-44CD-974B-54BFCD0DE856}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="0.29"/>
-        <filter val="-0.33"/>
-        <filter val="0.35"/>
-        <filter val="0.38"/>
-        <filter val="0.41"/>
-        <filter val="-0.41"/>
-        <filter val="0.48"/>
-        <filter val="-0.66"/>
-        <filter val="1.04"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:I139" xr:uid="{26FFD78D-BBF8-44CD-974B-54BFCD0DE856}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>